<commit_message>
adding DE ad and fs pages
</commit_message>
<xml_diff>
--- a/translations_slugs_excel.xlsx
+++ b/translations_slugs_excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j.roe.AD\Documents\Code\online-exerzitien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3377C97F-7E9E-497C-8A13-A707BA99F206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A191F02C-D2E6-46C0-ADD8-13EA96399837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,8 +19,19 @@
   <definedNames>
     <definedName name="ExterneDaten_1" localSheetId="0" hidden="1">translations_and_slugs_wide!$A$1:$Q$17</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -37,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="234">
   <si>
     <t>Column1</t>
   </si>
@@ -736,6 +747,9 @@
   </si>
   <si>
     <t>https://karmel.us6.list-manage.com/subscribe?u=7c9d2aa0ecc1fde64fd44bc67&amp;id=c32cba48a9</t>
+  </si>
+  <si>
+    <t>https://eepurl.us6.list-manage.com/subscribe?u=7c9d2aa0ecc1fde64fd44bc67&amp;id=48970c68bf</t>
   </si>
 </sst>
 </file>
@@ -1913,6 +1927,9 @@
       <c r="D16" t="s">
         <v>232</v>
       </c>
+      <c r="F16" s="4" t="s">
+        <v>233</v>
+      </c>
       <c r="H16" t="s">
         <v>231</v>
       </c>
@@ -1986,11 +2003,12 @@
     <hyperlink ref="P15" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
     <hyperlink ref="Q15" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
     <hyperlink ref="C16" r:id="rId11" xr:uid="{787A4DE5-335B-4B11-A6F3-1E6F83DC3CEE}"/>
+    <hyperlink ref="F16" r:id="rId12" xr:uid="{BCA7FA4C-37A2-4ED7-9F0D-002142A07A10}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId12"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId13"/>
   <tableParts count="1">
-    <tablePart r:id="rId13"/>
+    <tablePart r:id="rId14"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
changing current retreat to ./archive (DE)
</commit_message>
<xml_diff>
--- a/translations_slugs_excel.xlsx
+++ b/translations_slugs_excel.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j.roe.AD\Documents\Code\online-exerzitien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A191F02C-D2E6-46C0-ADD8-13EA96399837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B54F7EF3-FAC9-495E-AA3C-FD5B1BD556AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="translations_and_slugs_wide" sheetId="1" r:id="rId1"/>
     <sheet name="Tabelle1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="ExterneDaten_1" localSheetId="0" hidden="1">translations_and_slugs_wide!$A$1:$Q$17</definedName>
+    <definedName name="ExterneDaten_1" localSheetId="0" hidden="1">translations_and_slugs_wide!$A$1:$Q$55</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,10 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="234">
-  <si>
-    <t>Column1</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="312">
   <si>
     <t>Column2</t>
   </si>
@@ -101,9 +98,6 @@
     <t>Column17</t>
   </si>
   <si>
-    <t>word</t>
-  </si>
-  <si>
     <t>fr</t>
   </si>
   <si>
@@ -750,13 +744,258 @@
   </si>
   <si>
     <t>https://eepurl.us6.list-manage.com/subscribe?u=7c9d2aa0ecc1fde64fd44bc67&amp;id=48970c68bf</t>
+  </si>
+  <si>
+    <t>Eine Zeit der Besinnung, des Gebetes und der Erneuerung</t>
+  </si>
+  <si>
+    <t>hero-eyebrow</t>
+  </si>
+  <si>
+    <t>hero-h1</t>
+  </si>
+  <si>
+    <t>Online Exerzitien zur Advents- und Fastenzeit in der Schule der Heiligen des Karmel.</t>
+  </si>
+  <si>
+    <t>Erhalten Sie kostenlos die wöchentlichen Meditationen der Unbeschuhten Karmeliten</t>
+  </si>
+  <si>
+    <t>Anmeldung</t>
+  </si>
+  <si>
+    <t>signup-eyebrow</t>
+  </si>
+  <si>
+    <t>signup-h3</t>
+  </si>
+  <si>
+    <t>eMail Adresse* (erforderlich)</t>
+  </si>
+  <si>
+    <t>Vorname</t>
+  </si>
+  <si>
+    <t>Nachname</t>
+  </si>
+  <si>
+    <t>Wie sind Sie auf uns aufmerksam geworden?</t>
+  </si>
+  <si>
+    <t>HOWFOUND</t>
+  </si>
+  <si>
+    <t>Ja, ich melde mich an</t>
+  </si>
+  <si>
+    <t>signup-button</t>
+  </si>
+  <si>
+    <t>Datenschutz</t>
+  </si>
+  <si>
+    <t>Die Karmeliten in Österreich werden die Informationen, die Sie in diesem Formular angeben, dazu verwenden, mit Ihnen in Kontakt zu bleiben und Ihnen Informationen über Internet-Aktivitäten wie Exerzitien Online o.ä. zu übermitteln – je nach Ihrer Auswahl im obigen Formular. Sie können Ihre Meinung jederzeit ändern, indem Sie auf den Abbestellungs-Link klicken, den Sie in der Fußzeile jeder E-Mail, die Sie von uns erhalten, finden können, oder indem Sie uns unter online-exerzitien@karmel.at kontaktieren. Wir werden Ihre Informationen mit Sorgfalt und Respekt behandeln. Weitere Informationen zu unseren Datenschutzpraktiken finden Sie auf unserer Website www.karmel.at. Indem Sie unten klicken, erklären Sie sich damit einverstanden, dass wir Ihre Informationen in Übereinstimmung mit diesen Bedingungen verarbeiten dürfen.
+Wir nutzen Mailchimp als unsere Marketing-Plattform. Mit einem Klick auf den untenstehenden Button zum Abonnieren erklären Sie sich damit einverstanden, dass Ihre Daten zur Verarbeitung an Mailchimp übermittelt werden.</t>
+  </si>
+  <si>
+    <t>Mehr über die Datenschutzpraktiken von Mailchimp erfahren Sie hier.</t>
+  </si>
+  <si>
+    <t>privacy_title</t>
+  </si>
+  <si>
+    <t>privacy_desc</t>
+  </si>
+  <si>
+    <t>privacy_link</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Aktuelle Exerzitien</t>
+  </si>
+  <si>
+    <t>header_link_1</t>
+  </si>
+  <si>
+    <t>header_link_2</t>
+  </si>
+  <si>
+    <t>header_link_3</t>
+  </si>
+  <si>
+    <t>header_link_4</t>
+  </si>
+  <si>
+    <t>header_link_5</t>
+  </si>
+  <si>
+    <t>Vergangene Exerzitien</t>
+  </si>
+  <si>
+    <t>Wer sind wir?</t>
+  </si>
+  <si>
+    <t>Unterstützung</t>
+  </si>
+  <si>
+    <t>retreat_link</t>
+  </si>
+  <si>
+    <t>Mehr zu den Exerzitien</t>
+  </si>
+  <si>
+    <t>Inhalt</t>
+  </si>
+  <si>
+    <t>Jeden Freitag erhalten Sie eine E-Mail mit dem Folgenden:</t>
+  </si>
+  <si>
+    <t>Sie können den Text von dort aus herunterladen (in die folgenden Formate: A4 PDF und mobiloptimiertes PDF) oder die Audioversion als Podcast anhören. Der Inhalt der Betrachtung geht vom Sonntagsevangelium aus und führt uns in die Lehre des Heiligen ein. Ein Fastenkalender (Zitate und Bilder) wird Sie außerdem jeden Tag, von Montag bis Samstag, durch geistliche Impulse bereichern.</t>
+  </si>
+  <si>
+    <t>Ausgewählte Reihen der vergangenen Jahre</t>
+  </si>
+  <si>
+    <t>contents</t>
+  </si>
+  <si>
+    <t>contents_header</t>
+  </si>
+  <si>
+    <t>contents_info</t>
+  </si>
+  <si>
+    <t>archive_h2</t>
+  </si>
+  <si>
+    <t>load_more</t>
+  </si>
+  <si>
+    <t>Mehr laden</t>
+  </si>
+  <si>
+    <t>Die Spiritualität des Karmel lebt aus dem Zeugnis Mariens, der biblischen Gestalten des Karmel und vieler Heiliger, Seliger und geistlicher Lehrer.</t>
+  </si>
+  <si>
+    <t>saints_h3</t>
+  </si>
+  <si>
+    <t>Häufige Fragen</t>
+  </si>
+  <si>
+    <t>FAQ</t>
+  </si>
+  <si>
+    <t>Was sind Online-Exerzitien?</t>
+  </si>
+  <si>
+    <t>Online-Exerzitien sind geistliche Impulse, die per E-Mail verschickt werden und Sie durch Advent oder Fastenzeit begleiten.</t>
+  </si>
+  <si>
+    <t>Wie oft erhalte ich Nachrichten?</t>
+  </si>
+  <si>
+    <t>Sie erhalten zu Beginn eine Einführungsnachricht und danach regelmäßig weitere E-Mails während der jeweiligen Exerzitienzeit.</t>
+  </si>
+  <si>
+    <t>Ist die Teilnahme kostenpflichtig?</t>
+  </si>
+  <si>
+    <t>Die Anmeldung ist kostenlos. Eine freiwillige Spende kann zur Unterstützung des Apostolats vorgesehen sein.</t>
+  </si>
+  <si>
+    <t>Ich bekomme keine E-Mails – was tun?</t>
+  </si>
+  <si>
+    <t>Bitte prüfen Sie Ihren Spam-Ordner sowie gegebenenfalls den Reiter „Werbung“ oder „Promotionen“ in Ihrem E-Mail-Postfach.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Laden Sie auch Freunde und Bekannte ein! Sie können diese Seite weiterempfehlen oder auf online-exerzitien.karmel.at verweisen.
+Wenn Sie sich mit dem online-Anmeldeformular schwer tun oder Fehler auftreten, schreiben Sie uns ein eMail.
+Sie können die Exerzitien/Novenen und die anderen Aussendungen auch über die kostenlose App "Gott allein genügt!" für iPhone, Android und Windows Mobile verfolgen: Homepage der App - dort finden Sie auch weitere Impulse und Infos.
+So wünschen wir Ihnen ein gutes, frohes Lesen und Beten! </t>
+  </si>
+  <si>
+    <t>Plakat (A4)</t>
+  </si>
+  <si>
+    <t>Die Karmeliten danken Ihnen für jede Spende, mit der Sie die technische Umsetzung der Exerzitien unterstützen!</t>
+  </si>
+  <si>
+    <t>Sie können Ihre Spende an folgendes Konto:
+Karmeliten in Österreich</t>
+  </si>
+  <si>
+    <t>Spenden</t>
+  </si>
+  <si>
+    <t>EN:</t>
+  </si>
+  <si>
+    <t>DE:</t>
+  </si>
+  <si>
+    <t>FR:</t>
+  </si>
+  <si>
+    <t>language code</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>firstname</t>
+  </si>
+  <si>
+    <t>lastname</t>
+  </si>
+  <si>
+    <t>what_a</t>
+  </si>
+  <si>
+    <t>what_q</t>
+  </si>
+  <si>
+    <t>when_q</t>
+  </si>
+  <si>
+    <t>when_a</t>
+  </si>
+  <si>
+    <t>cost_q</t>
+  </si>
+  <si>
+    <t>cost_a</t>
+  </si>
+  <si>
+    <t>problem_q</t>
+  </si>
+  <si>
+    <t>problem_a</t>
+  </si>
+  <si>
+    <t>invite</t>
+  </si>
+  <si>
+    <t>poster</t>
+  </si>
+  <si>
+    <t>donate</t>
+  </si>
+  <si>
+    <t>donate_p</t>
+  </si>
+  <si>
+    <t>donate_p2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -784,6 +1023,12 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -806,12 +1051,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -899,15 +1147,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="translations_and_slugs_wide" displayName="translations_and_slugs_wide" ref="A1:Q17" totalsRowShown="0">
-  <autoFilter ref="A1:Q17" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="translations_and_slugs_wide" displayName="translations_and_slugs_wide" ref="A1:Q55" totalsRowShown="0">
+  <autoFilter ref="A1:Q55" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Column1"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Column2"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Column3"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Column4"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Column5"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Column6"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Column2"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Column7"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Column8"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Column9"/>
@@ -1100,31 +1348,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" customWidth="1"/>
-    <col min="2" max="2" width="15.5703125" customWidth="1"/>
-    <col min="3" max="3" width="22.85546875" customWidth="1"/>
+    <col min="3" max="3" width="36.7109375" customWidth="1"/>
     <col min="4" max="4" width="20.140625" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
     <col min="6" max="6" width="19.7109375" customWidth="1"/>
-    <col min="7" max="7" width="16.5703125" customWidth="1"/>
-    <col min="8" max="8" width="18.85546875" customWidth="1"/>
-    <col min="9" max="9" width="20.28515625" customWidth="1"/>
-    <col min="10" max="10" width="18.7109375" customWidth="1"/>
-    <col min="11" max="11" width="22.28515625" customWidth="1"/>
-    <col min="12" max="12" width="20.7109375" customWidth="1"/>
-    <col min="13" max="13" width="19.28515625" customWidth="1"/>
-    <col min="14" max="14" width="17" customWidth="1"/>
-    <col min="15" max="15" width="24.85546875" customWidth="1"/>
-    <col min="16" max="16" width="16.7109375" customWidth="1"/>
-    <col min="17" max="17" width="23.5703125" customWidth="1"/>
+    <col min="7" max="7" width="15.5703125" customWidth="1"/>
+    <col min="8" max="8" width="16.5703125" customWidth="1"/>
+    <col min="9" max="9" width="18.85546875" customWidth="1"/>
+    <col min="10" max="10" width="20.28515625" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" customWidth="1"/>
+    <col min="12" max="12" width="22.28515625" customWidth="1"/>
+    <col min="13" max="13" width="20.7109375" customWidth="1"/>
+    <col min="14" max="14" width="19.28515625" customWidth="1"/>
+    <col min="15" max="15" width="17" customWidth="1"/>
+    <col min="16" max="16" width="24.85546875" customWidth="1"/>
+    <col min="17" max="17" width="16.7109375" customWidth="1"/>
+    <col min="18" max="18" width="23.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -1139,860 +1387,1165 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>15</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>295</v>
+      </c>
+      <c r="B2" t="s">
         <v>17</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>18</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>19</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>20</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" t="s">
         <v>21</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>22</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>23</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>24</v>
       </c>
-      <c r="I2" t="s">
+      <c r="K2" t="s">
         <v>25</v>
       </c>
-      <c r="J2" t="s">
+      <c r="L2" t="s">
         <v>26</v>
       </c>
-      <c r="K2" t="s">
+      <c r="M2" t="s">
         <v>27</v>
       </c>
-      <c r="L2" t="s">
+      <c r="N2" t="s">
         <v>28</v>
       </c>
-      <c r="M2" t="s">
+      <c r="O2" t="s">
         <v>29</v>
       </c>
-      <c r="N2" t="s">
+      <c r="P2" t="s">
         <v>30</v>
       </c>
-      <c r="O2" t="s">
+      <c r="Q2" t="s">
         <v>31</v>
-      </c>
-      <c r="P2" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
         <v>34</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>34</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" t="s">
         <v>35</v>
       </c>
-      <c r="D3" t="s">
+      <c r="H3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="I3" t="s">
         <v>34</v>
       </c>
-      <c r="G3" t="s">
+      <c r="J3" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="K3" t="s">
         <v>38</v>
       </c>
-      <c r="I3" t="s">
-        <v>36</v>
-      </c>
-      <c r="J3" s="2" t="s">
+      <c r="L3" t="s">
         <v>39</v>
       </c>
-      <c r="K3" t="s">
+      <c r="M3" t="s">
         <v>40</v>
       </c>
-      <c r="L3" t="s">
+      <c r="N3" t="s">
         <v>41</v>
       </c>
-      <c r="M3" t="s">
+      <c r="O3" t="s">
         <v>42</v>
       </c>
-      <c r="N3" t="s">
+      <c r="P3" t="s">
         <v>43</v>
       </c>
-      <c r="O3" t="s">
+      <c r="Q3" t="s">
         <v>44</v>
-      </c>
-      <c r="P3" t="s">
-        <v>45</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" t="s">
         <v>47</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" t="s">
+        <v>49</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I4" t="s">
         <v>47</v>
       </c>
-      <c r="C4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D4" t="s">
-        <v>49</v>
-      </c>
-      <c r="E4" t="s">
-        <v>50</v>
-      </c>
-      <c r="F4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="J4" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="K4" t="s">
         <v>52</v>
       </c>
-      <c r="I4" t="s">
-        <v>49</v>
-      </c>
-      <c r="J4" s="2" t="s">
+      <c r="L4" t="s">
+        <v>39</v>
+      </c>
+      <c r="M4" t="s">
         <v>53</v>
       </c>
-      <c r="K4" t="s">
+      <c r="N4" t="s">
         <v>54</v>
       </c>
-      <c r="L4" t="s">
-        <v>41</v>
-      </c>
-      <c r="M4" t="s">
+      <c r="O4" t="s">
         <v>55</v>
       </c>
-      <c r="N4" t="s">
+      <c r="P4" t="s">
         <v>56</v>
       </c>
-      <c r="O4" t="s">
+      <c r="Q4" t="s">
         <v>57</v>
-      </c>
-      <c r="P4" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" t="s">
         <v>60</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>61</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>62</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" t="s">
         <v>63</v>
       </c>
-      <c r="E5" t="s">
+      <c r="H5" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="F5" t="s">
-        <v>60</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="I5" t="s">
         <v>65</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="J5" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="I5" t="s">
+      <c r="K5" t="s">
         <v>67</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="L5" t="s">
         <v>68</v>
       </c>
-      <c r="K5" t="s">
+      <c r="M5" t="s">
         <v>69</v>
       </c>
-      <c r="L5" t="s">
+      <c r="N5" t="s">
         <v>70</v>
       </c>
-      <c r="M5" t="s">
+      <c r="O5" t="s">
         <v>71</v>
       </c>
-      <c r="N5" t="s">
+      <c r="P5" t="s">
         <v>72</v>
       </c>
-      <c r="O5" t="s">
+      <c r="Q5" t="s">
         <v>73</v>
-      </c>
-      <c r="P5" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" t="s">
         <v>76</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>77</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>78</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>79</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
+        <v>75</v>
+      </c>
+      <c r="G6" t="s">
         <v>80</v>
       </c>
-      <c r="F6" t="s">
+      <c r="H6" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="G6" t="s">
+      <c r="I6" t="s">
         <v>82</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="J6" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="I6" t="s">
+      <c r="K6" t="s">
         <v>84</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="L6" t="s">
         <v>85</v>
       </c>
-      <c r="K6" t="s">
+      <c r="M6" t="s">
         <v>86</v>
       </c>
-      <c r="L6" t="s">
+      <c r="N6" t="s">
         <v>87</v>
       </c>
-      <c r="M6" t="s">
+      <c r="O6" t="s">
         <v>88</v>
       </c>
-      <c r="N6" t="s">
+      <c r="P6" t="s">
         <v>89</v>
       </c>
-      <c r="O6" t="s">
+      <c r="Q6" t="s">
         <v>90</v>
-      </c>
-      <c r="P6" t="s">
-        <v>91</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B7" t="s">
         <v>93</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>94</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>95</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
+        <v>93</v>
+      </c>
+      <c r="F7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G7" t="s">
         <v>96</v>
       </c>
-      <c r="E7" t="s">
+      <c r="H7" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="F7" t="s">
-        <v>95</v>
-      </c>
-      <c r="G7" t="s">
+      <c r="I7" t="s">
         <v>98</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="J7" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="I7" t="s">
+      <c r="K7" t="s">
+        <v>93</v>
+      </c>
+      <c r="L7" t="s">
         <v>100</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="M7" t="s">
+        <v>93</v>
+      </c>
+      <c r="N7" t="s">
         <v>101</v>
       </c>
-      <c r="K7" t="s">
-        <v>95</v>
-      </c>
-      <c r="L7" t="s">
+      <c r="O7" t="s">
+        <v>93</v>
+      </c>
+      <c r="P7" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q7" t="s">
         <v>102</v>
-      </c>
-      <c r="M7" t="s">
-        <v>95</v>
-      </c>
-      <c r="N7" t="s">
-        <v>103</v>
-      </c>
-      <c r="O7" t="s">
-        <v>95</v>
-      </c>
-      <c r="P7" t="s">
-        <v>95</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" t="s">
         <v>105</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>106</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>107</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>108</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
+        <v>104</v>
+      </c>
+      <c r="G8" t="s">
         <v>109</v>
       </c>
-      <c r="F8" t="s">
+      <c r="H8" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="G8" t="s">
+      <c r="I8" t="s">
+        <v>106</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="K8" t="s">
         <v>112</v>
       </c>
-      <c r="I8" t="s">
-        <v>108</v>
-      </c>
-      <c r="J8" s="2" t="s">
+      <c r="L8" t="s">
         <v>113</v>
       </c>
-      <c r="K8" t="s">
+      <c r="M8" t="s">
         <v>114</v>
       </c>
-      <c r="L8" t="s">
+      <c r="N8" t="s">
         <v>115</v>
       </c>
-      <c r="M8" t="s">
+      <c r="O8" t="s">
         <v>116</v>
       </c>
-      <c r="N8" t="s">
+      <c r="P8" t="s">
         <v>117</v>
       </c>
-      <c r="O8" t="s">
+      <c r="Q8" t="s">
         <v>118</v>
-      </c>
-      <c r="P8" t="s">
-        <v>119</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B9" t="s">
         <v>121</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>122</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>123</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>124</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
+        <v>120</v>
+      </c>
+      <c r="G9" t="s">
         <v>125</v>
       </c>
-      <c r="F9" t="s">
+      <c r="H9" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="G9" t="s">
+      <c r="I9" t="s">
         <v>127</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="J9" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="I9" t="s">
+      <c r="K9" t="s">
         <v>129</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="L9" t="s">
         <v>130</v>
       </c>
-      <c r="K9" t="s">
+      <c r="M9" t="s">
         <v>131</v>
       </c>
-      <c r="L9" t="s">
+      <c r="N9" t="s">
         <v>132</v>
       </c>
-      <c r="M9" t="s">
+      <c r="O9" t="s">
         <v>133</v>
       </c>
-      <c r="N9" t="s">
+      <c r="P9" t="s">
         <v>134</v>
       </c>
-      <c r="O9" t="s">
+      <c r="Q9" t="s">
         <v>135</v>
-      </c>
-      <c r="P9" t="s">
-        <v>136</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B10" t="s">
         <v>138</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>139</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>140</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>141</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
+        <v>137</v>
+      </c>
+      <c r="G10" t="s">
         <v>142</v>
       </c>
-      <c r="F10" t="s">
+      <c r="H10" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="G10" t="s">
+      <c r="I10" t="s">
         <v>144</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="J10" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="I10" t="s">
+      <c r="K10" t="s">
         <v>146</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="L10" t="s">
         <v>147</v>
       </c>
-      <c r="K10" t="s">
+      <c r="M10" t="s">
         <v>148</v>
       </c>
-      <c r="L10" t="s">
+      <c r="N10" t="s">
         <v>149</v>
       </c>
-      <c r="M10" t="s">
+      <c r="O10" t="s">
         <v>150</v>
       </c>
-      <c r="N10" t="s">
+      <c r="P10" t="s">
         <v>151</v>
       </c>
-      <c r="O10" t="s">
+      <c r="Q10" t="s">
         <v>152</v>
-      </c>
-      <c r="P10" t="s">
-        <v>153</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>153</v>
+      </c>
+      <c r="B11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" t="s">
+        <v>154</v>
+      </c>
+      <c r="H11" t="s">
         <v>155</v>
       </c>
-      <c r="B11" t="s">
+      <c r="I11" t="s">
         <v>47</v>
       </c>
-      <c r="C11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" t="s">
-        <v>49</v>
-      </c>
-      <c r="E11" t="s">
-        <v>50</v>
-      </c>
-      <c r="F11" t="s">
-        <v>47</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="J11" t="s">
         <v>156</v>
       </c>
-      <c r="H11" t="s">
+      <c r="K11" t="s">
         <v>157</v>
       </c>
-      <c r="I11" t="s">
-        <v>49</v>
-      </c>
-      <c r="J11" t="s">
+      <c r="L11" t="s">
+        <v>39</v>
+      </c>
+      <c r="M11" t="s">
+        <v>53</v>
+      </c>
+      <c r="N11" t="s">
+        <v>54</v>
+      </c>
+      <c r="O11" t="s">
+        <v>55</v>
+      </c>
+      <c r="P11" t="s">
         <v>158</v>
       </c>
-      <c r="K11" t="s">
+      <c r="Q11" t="s">
         <v>159</v>
-      </c>
-      <c r="L11" t="s">
-        <v>41</v>
-      </c>
-      <c r="M11" t="s">
-        <v>55</v>
-      </c>
-      <c r="N11" t="s">
-        <v>56</v>
-      </c>
-      <c r="O11" t="s">
-        <v>57</v>
-      </c>
-      <c r="P11" t="s">
-        <v>160</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>160</v>
+      </c>
+      <c r="B12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" t="s">
+        <v>61</v>
+      </c>
+      <c r="D12" t="s">
+        <v>62</v>
+      </c>
+      <c r="E12" t="s">
+        <v>58</v>
+      </c>
+      <c r="F12" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" t="s">
+        <v>63</v>
+      </c>
+      <c r="H12" t="s">
+        <v>161</v>
+      </c>
+      <c r="I12" t="s">
+        <v>65</v>
+      </c>
+      <c r="J12" t="s">
         <v>162</v>
       </c>
-      <c r="B12" t="s">
-        <v>61</v>
-      </c>
-      <c r="C12" t="s">
-        <v>69</v>
-      </c>
-      <c r="D12" t="s">
-        <v>63</v>
-      </c>
-      <c r="E12" t="s">
-        <v>64</v>
-      </c>
-      <c r="F12" t="s">
-        <v>60</v>
-      </c>
-      <c r="G12" t="s">
-        <v>65</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="K12" t="s">
+        <v>67</v>
+      </c>
+      <c r="L12" t="s">
+        <v>68</v>
+      </c>
+      <c r="M12" t="s">
         <v>163</v>
       </c>
-      <c r="I12" t="s">
-        <v>67</v>
-      </c>
-      <c r="J12" t="s">
+      <c r="N12" t="s">
+        <v>70</v>
+      </c>
+      <c r="O12" t="s">
+        <v>71</v>
+      </c>
+      <c r="P12" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q12" t="s">
         <v>164</v>
-      </c>
-      <c r="K12" t="s">
-        <v>69</v>
-      </c>
-      <c r="L12" t="s">
-        <v>70</v>
-      </c>
-      <c r="M12" t="s">
-        <v>165</v>
-      </c>
-      <c r="N12" t="s">
-        <v>72</v>
-      </c>
-      <c r="O12" t="s">
-        <v>73</v>
-      </c>
-      <c r="P12" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>165</v>
+      </c>
+      <c r="B13" t="s">
         <v>167</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>168</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>169</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" t="s">
+        <v>166</v>
+      </c>
+      <c r="G13" t="s">
         <v>170</v>
       </c>
-      <c r="E13" t="s">
+      <c r="H13" t="s">
         <v>171</v>
       </c>
-      <c r="F13" t="s">
-        <v>76</v>
-      </c>
-      <c r="G13" t="s">
+      <c r="I13" t="s">
         <v>172</v>
       </c>
-      <c r="H13" t="s">
+      <c r="J13" t="s">
         <v>173</v>
       </c>
-      <c r="I13" t="s">
+      <c r="K13" t="s">
         <v>174</v>
       </c>
-      <c r="J13" t="s">
+      <c r="L13" t="s">
         <v>175</v>
       </c>
-      <c r="K13" t="s">
+      <c r="M13" t="s">
         <v>176</v>
       </c>
-      <c r="L13" t="s">
+      <c r="N13" t="s">
         <v>177</v>
       </c>
-      <c r="M13" t="s">
+      <c r="O13" t="s">
         <v>178</v>
       </c>
-      <c r="N13" t="s">
+      <c r="P13" t="s">
         <v>179</v>
       </c>
-      <c r="O13" t="s">
+      <c r="Q13" t="s">
         <v>180</v>
-      </c>
-      <c r="P13" t="s">
-        <v>181</v>
-      </c>
-      <c r="Q13" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B14" t="s">
+        <v>91</v>
+      </c>
+      <c r="C14" t="s">
         <v>183</v>
       </c>
-      <c r="B14" t="s">
+      <c r="D14" t="s">
         <v>184</v>
       </c>
-      <c r="C14" t="s">
-        <v>93</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
+        <v>91</v>
+      </c>
+      <c r="F14" t="s">
+        <v>182</v>
+      </c>
+      <c r="G14" t="s">
         <v>185</v>
       </c>
-      <c r="E14" t="s">
+      <c r="H14" t="s">
         <v>186</v>
       </c>
-      <c r="F14" t="s">
-        <v>93</v>
-      </c>
-      <c r="G14" t="s">
+      <c r="I14" t="s">
         <v>187</v>
       </c>
-      <c r="H14" t="s">
+      <c r="J14" t="s">
         <v>188</v>
       </c>
-      <c r="I14" t="s">
+      <c r="K14" t="s">
+        <v>91</v>
+      </c>
+      <c r="L14" t="s">
         <v>189</v>
       </c>
-      <c r="J14" t="s">
+      <c r="M14" t="s">
+        <v>91</v>
+      </c>
+      <c r="N14" t="s">
         <v>190</v>
       </c>
-      <c r="K14" t="s">
-        <v>93</v>
-      </c>
-      <c r="L14" t="s">
+      <c r="O14" t="s">
+        <v>91</v>
+      </c>
+      <c r="P14" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q14" t="s">
         <v>191</v>
-      </c>
-      <c r="M14" t="s">
-        <v>93</v>
-      </c>
-      <c r="N14" t="s">
-        <v>192</v>
-      </c>
-      <c r="O14" t="s">
-        <v>93</v>
-      </c>
-      <c r="P14" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q14" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>192</v>
+      </c>
+      <c r="B15" t="s">
         <v>194</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>195</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>196</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>197</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
+        <v>193</v>
+      </c>
+      <c r="G15" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="F15" t="s">
+      <c r="H15" t="s">
         <v>199</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="I15" t="s">
         <v>200</v>
       </c>
-      <c r="H15" t="s">
+      <c r="J15" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="I15" t="s">
+      <c r="K15" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="J15" s="3" t="s">
+      <c r="L15" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="K15" s="3" t="s">
+      <c r="M15" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="L15" s="3" t="s">
+      <c r="N15" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="M15" s="3" t="s">
+      <c r="O15" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="N15" s="3" t="s">
+      <c r="P15" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="O15" s="3" t="s">
+      <c r="Q15" s="3" t="s">
         <v>208</v>
-      </c>
-      <c r="P15" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="Q15" s="3" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>211</v>
-      </c>
-      <c r="C16" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="C16" t="s">
         <v>230</v>
       </c>
-      <c r="D16" t="s">
-        <v>232</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>233</v>
+      <c r="E16" s="4" t="s">
+        <v>231</v>
       </c>
       <c r="H16" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="L16" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="N16" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>210</v>
+      </c>
+      <c r="B17" t="s">
+        <v>211</v>
+      </c>
+      <c r="C17" t="s">
         <v>212</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>213</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>214</v>
       </c>
-      <c r="E17" t="s">
+      <c r="G17" t="s">
         <v>215</v>
       </c>
-      <c r="F17" t="s">
+      <c r="H17" t="s">
         <v>216</v>
       </c>
-      <c r="G17" t="s">
+      <c r="I17" t="s">
         <v>217</v>
       </c>
-      <c r="H17" t="s">
+      <c r="J17" t="s">
         <v>218</v>
       </c>
-      <c r="I17" t="s">
+      <c r="K17" t="s">
         <v>219</v>
       </c>
-      <c r="J17" t="s">
+      <c r="L17" t="s">
         <v>220</v>
       </c>
-      <c r="K17" t="s">
+      <c r="M17" t="s">
         <v>221</v>
       </c>
-      <c r="L17" t="s">
+      <c r="N17" t="s">
         <v>222</v>
       </c>
-      <c r="M17" t="s">
+      <c r="O17" t="s">
         <v>223</v>
       </c>
-      <c r="N17" t="s">
+      <c r="P17" t="s">
         <v>224</v>
       </c>
-      <c r="O17" t="s">
+      <c r="Q17" t="s">
         <v>225</v>
       </c>
-      <c r="P17" t="s">
-        <v>226</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>227</v>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>255</v>
+      </c>
+      <c r="B18" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>256</v>
+      </c>
+      <c r="B19" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>257</v>
+      </c>
+      <c r="B20" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>258</v>
+      </c>
+      <c r="B21" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>259</v>
+      </c>
+      <c r="B22" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>233</v>
+      </c>
+      <c r="B23" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>234</v>
+      </c>
+      <c r="B24" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>239</v>
+      </c>
+      <c r="B25" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>238</v>
+      </c>
+      <c r="B26" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>296</v>
+      </c>
+      <c r="B27" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>297</v>
+      </c>
+      <c r="B28" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>298</v>
+      </c>
+      <c r="B29" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>244</v>
+      </c>
+      <c r="B30" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>246</v>
+      </c>
+      <c r="B31" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>250</v>
+      </c>
+      <c r="B32" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>251</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>252</v>
+      </c>
+      <c r="B34" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>263</v>
+      </c>
+      <c r="B35" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>269</v>
+      </c>
+      <c r="B36" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>270</v>
+      </c>
+      <c r="B37" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>271</v>
+      </c>
+      <c r="B38" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>272</v>
+      </c>
+      <c r="B39" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>273</v>
+      </c>
+      <c r="B40" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>276</v>
+      </c>
+      <c r="B41" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>278</v>
+      </c>
+      <c r="B42" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>300</v>
+      </c>
+      <c r="B43" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>299</v>
+      </c>
+      <c r="B44" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>301</v>
+      </c>
+      <c r="B45" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>302</v>
+      </c>
+      <c r="B46" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>303</v>
+      </c>
+      <c r="B47" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>304</v>
+      </c>
+      <c r="B48" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>305</v>
+      </c>
+      <c r="B49" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>306</v>
+      </c>
+      <c r="B50" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>307</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>308</v>
+      </c>
+      <c r="B52" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>309</v>
+      </c>
+      <c r="B53" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>310</v>
+      </c>
+      <c r="B54" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" ht="135" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>311</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="C15" r:id="rId1" display="https://exerzitien" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="B15" r:id="rId1" display="https://exerzitien" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="G15" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="J15" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
     <hyperlink ref="K15" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
@@ -2002,8 +2555,8 @@
     <hyperlink ref="O15" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
     <hyperlink ref="P15" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
     <hyperlink ref="Q15" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="C16" r:id="rId11" xr:uid="{787A4DE5-335B-4B11-A6F3-1E6F83DC3CEE}"/>
-    <hyperlink ref="F16" r:id="rId12" xr:uid="{BCA7FA4C-37A2-4ED7-9F0D-002142A07A10}"/>
+    <hyperlink ref="B16" r:id="rId11" xr:uid="{787A4DE5-335B-4B11-A6F3-1E6F83DC3CEE}"/>
+    <hyperlink ref="E16" r:id="rId12" xr:uid="{BCA7FA4C-37A2-4ED7-9F0D-002142A07A10}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId13"/>
@@ -2015,9 +2568,25 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A2:A4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>294</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
adding Indonesian removing old translations file
</commit_message>
<xml_diff>
--- a/translations_slugs_excel.xlsx
+++ b/translations_slugs_excel.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j.roe.AD\Documents\Code\online-exerzitien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B54F7EF3-FAC9-495E-AA3C-FD5B1BD556AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBA7F243-E33F-4B8D-BEB3-516E750BE86B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="translations_and_slugs_wide" sheetId="1" r:id="rId1"/>
     <sheet name="Tabelle1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="ExterneDaten_1" localSheetId="0" hidden="1">translations_and_slugs_wide!$A$1:$Q$55</definedName>
+    <definedName name="ExterneDaten_1" localSheetId="0" hidden="1">translations_and_slugs_wide!$A$1:$Q$56</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="317">
   <si>
     <t>Column2</t>
   </si>
@@ -678,9 +678,6 @@
   </si>
   <si>
     <t>mailchimp (old)</t>
-  </si>
-  <si>
-    <t>prefix</t>
   </si>
   <si>
     <t>exerzitien-online</t>
@@ -989,6 +986,24 @@
   </si>
   <si>
     <t>donate_p2</t>
+  </si>
+  <si>
+    <t>subdomain</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>Column18</t>
+  </si>
+  <si>
+    <t>language name Deutsch</t>
+  </si>
+  <si>
+    <t>http://www.retret-online.karmel.at/</t>
+  </si>
+  <si>
+    <t>retret-online</t>
   </si>
 </sst>
 </file>
@@ -1147,9 +1162,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="translations_and_slugs_wide" displayName="translations_and_slugs_wide" ref="A1:Q55" totalsRowShown="0">
-  <autoFilter ref="A1:Q55" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="translations_and_slugs_wide" displayName="translations_and_slugs_wide" ref="A1:R56" totalsRowShown="0">
+  <autoFilter ref="A1:R56" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Column3"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Column4"/>
@@ -1167,6 +1182,7 @@
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Column15"/>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Column16"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Column17"/>
+    <tableColumn id="18" xr3:uid="{8B8DFB27-EECB-4AA6-AFA9-67F0D2F0D095}" name="Column18"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1348,7 +1364,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q55"/>
+  <dimension ref="A1:R56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" customWidth="1"/>
@@ -1370,9 +1386,9 @@
     <col min="18" max="18" width="23.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -1422,10 +1438,13 @@
       <c r="Q1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R1" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B2" t="s">
         <v>17</v>
@@ -1475,975 +1494,981 @@
       <c r="Q2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="R2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>32</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>33</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>34</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D4" t="s">
         <v>34</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E4" t="s">
         <v>32</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F4" t="s">
         <v>32</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G4" t="s">
         <v>35</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I4" t="s">
         <v>34</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K4" t="s">
         <v>38</v>
-      </c>
-      <c r="L3" t="s">
-        <v>39</v>
-      </c>
-      <c r="M3" t="s">
-        <v>40</v>
-      </c>
-      <c r="N3" t="s">
-        <v>41</v>
-      </c>
-      <c r="O3" t="s">
-        <v>42</v>
-      </c>
-      <c r="P3" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D4" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" t="s">
-        <v>45</v>
-      </c>
-      <c r="F4" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" t="s">
-        <v>49</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="I4" t="s">
-        <v>47</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="K4" t="s">
-        <v>52</v>
       </c>
       <c r="L4" t="s">
         <v>39</v>
       </c>
       <c r="M4" t="s">
+        <v>40</v>
+      </c>
+      <c r="N4" t="s">
+        <v>41</v>
+      </c>
+      <c r="O4" t="s">
+        <v>42</v>
+      </c>
+      <c r="P4" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F5" t="s">
+        <v>45</v>
+      </c>
+      <c r="G5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I5" t="s">
+        <v>47</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="K5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L5" t="s">
+        <v>39</v>
+      </c>
+      <c r="M5" t="s">
         <v>53</v>
       </c>
-      <c r="N4" t="s">
+      <c r="N5" t="s">
         <v>54</v>
       </c>
-      <c r="O4" t="s">
+      <c r="O5" t="s">
         <v>55</v>
       </c>
-      <c r="P4" t="s">
+      <c r="P5" t="s">
         <v>56</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="Q5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    <row r="6" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>58</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>60</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C6" t="s">
         <v>61</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D6" t="s">
         <v>62</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E6" t="s">
         <v>58</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F6" t="s">
         <v>59</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G6" t="s">
         <v>63</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I6" t="s">
         <v>65</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K6" t="s">
         <v>67</v>
       </c>
-      <c r="L5" t="s">
+      <c r="L6" t="s">
         <v>68</v>
       </c>
-      <c r="M5" t="s">
+      <c r="M6" t="s">
         <v>69</v>
       </c>
-      <c r="N5" t="s">
+      <c r="N6" t="s">
         <v>70</v>
       </c>
-      <c r="O5" t="s">
+      <c r="O6" t="s">
         <v>71</v>
       </c>
-      <c r="P5" t="s">
+      <c r="P6" t="s">
         <v>72</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="Q6" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+    <row r="7" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>74</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
         <v>76</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
         <v>77</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D7" t="s">
         <v>78</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E7" t="s">
         <v>79</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G7" t="s">
         <v>80</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I7" t="s">
         <v>82</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="J7" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="K6" t="s">
+      <c r="K7" t="s">
         <v>84</v>
       </c>
-      <c r="L6" t="s">
+      <c r="L7" t="s">
         <v>85</v>
       </c>
-      <c r="M6" t="s">
+      <c r="M7" t="s">
         <v>86</v>
       </c>
-      <c r="N6" t="s">
+      <c r="N7" t="s">
         <v>87</v>
       </c>
-      <c r="O6" t="s">
+      <c r="O7" t="s">
         <v>88</v>
       </c>
-      <c r="P6" t="s">
+      <c r="P7" t="s">
         <v>89</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="Q7" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+    <row r="8" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>91</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>93</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C8" t="s">
         <v>94</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D8" t="s">
         <v>95</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E8" t="s">
         <v>93</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F8" t="s">
         <v>92</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G8" t="s">
         <v>96</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I8" t="s">
         <v>98</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J8" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="K7" t="s">
+      <c r="K8" t="s">
         <v>93</v>
       </c>
-      <c r="L7" t="s">
+      <c r="L8" t="s">
         <v>100</v>
       </c>
-      <c r="M7" t="s">
+      <c r="M8" t="s">
         <v>93</v>
       </c>
-      <c r="N7" t="s">
+      <c r="N8" t="s">
         <v>101</v>
       </c>
-      <c r="O7" t="s">
+      <c r="O8" t="s">
         <v>93</v>
       </c>
-      <c r="P7" t="s">
+      <c r="P8" t="s">
         <v>93</v>
       </c>
-      <c r="Q7" t="s">
+      <c r="Q8" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+    <row r="9" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>103</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B9" t="s">
         <v>105</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C9" t="s">
         <v>106</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D9" t="s">
         <v>107</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E9" t="s">
         <v>108</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F9" t="s">
         <v>104</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G9" t="s">
         <v>109</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I9" t="s">
         <v>106</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="K8" t="s">
+      <c r="K9" t="s">
         <v>112</v>
       </c>
-      <c r="L8" t="s">
+      <c r="L9" t="s">
         <v>113</v>
       </c>
-      <c r="M8" t="s">
+      <c r="M9" t="s">
         <v>114</v>
       </c>
-      <c r="N8" t="s">
+      <c r="N9" t="s">
         <v>115</v>
       </c>
-      <c r="O8" t="s">
+      <c r="O9" t="s">
         <v>116</v>
       </c>
-      <c r="P8" t="s">
+      <c r="P9" t="s">
         <v>117</v>
       </c>
-      <c r="Q8" t="s">
+      <c r="Q9" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+    <row r="10" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>119</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
         <v>121</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C10" t="s">
         <v>122</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D10" t="s">
         <v>123</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E10" t="s">
         <v>124</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F10" t="s">
         <v>120</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G10" t="s">
         <v>125</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I10" t="s">
         <v>127</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J10" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K10" t="s">
         <v>129</v>
       </c>
-      <c r="L9" t="s">
+      <c r="L10" t="s">
         <v>130</v>
       </c>
-      <c r="M9" t="s">
+      <c r="M10" t="s">
         <v>131</v>
       </c>
-      <c r="N9" t="s">
+      <c r="N10" t="s">
         <v>132</v>
       </c>
-      <c r="O9" t="s">
+      <c r="O10" t="s">
         <v>133</v>
       </c>
-      <c r="P9" t="s">
+      <c r="P10" t="s">
         <v>134</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="Q10" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="11" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>136</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B11" t="s">
         <v>138</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C11" t="s">
         <v>139</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D11" t="s">
         <v>140</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E11" t="s">
         <v>141</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F11" t="s">
         <v>137</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G11" t="s">
         <v>142</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I11" t="s">
         <v>144</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="K10" t="s">
+      <c r="K11" t="s">
         <v>146</v>
       </c>
-      <c r="L10" t="s">
+      <c r="L11" t="s">
         <v>147</v>
       </c>
-      <c r="M10" t="s">
+      <c r="M11" t="s">
         <v>148</v>
       </c>
-      <c r="N10" t="s">
+      <c r="N11" t="s">
         <v>149</v>
       </c>
-      <c r="O10" t="s">
+      <c r="O11" t="s">
         <v>150</v>
       </c>
-      <c r="P10" t="s">
+      <c r="P11" t="s">
         <v>151</v>
       </c>
-      <c r="Q10" t="s">
+      <c r="Q11" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>153</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>42</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C12" t="s">
         <v>47</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D12" t="s">
         <v>48</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E12" t="s">
         <v>45</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F12" t="s">
         <v>45</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G12" t="s">
         <v>154</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H12" t="s">
         <v>155</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I12" t="s">
         <v>47</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J12" t="s">
         <v>156</v>
       </c>
-      <c r="K11" t="s">
+      <c r="K12" t="s">
         <v>157</v>
       </c>
-      <c r="L11" t="s">
+      <c r="L12" t="s">
         <v>39</v>
       </c>
-      <c r="M11" t="s">
+      <c r="M12" t="s">
         <v>53</v>
       </c>
-      <c r="N11" t="s">
+      <c r="N12" t="s">
         <v>54</v>
       </c>
-      <c r="O11" t="s">
+      <c r="O12" t="s">
         <v>55</v>
       </c>
-      <c r="P11" t="s">
+      <c r="P12" t="s">
         <v>158</v>
       </c>
-      <c r="Q11" t="s">
+      <c r="Q12" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>160</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
         <v>67</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C13" t="s">
         <v>61</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D13" t="s">
         <v>62</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E13" t="s">
         <v>58</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F13" t="s">
         <v>59</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G13" t="s">
         <v>63</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H13" t="s">
         <v>161</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I13" t="s">
         <v>65</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J13" t="s">
         <v>162</v>
       </c>
-      <c r="K12" t="s">
+      <c r="K13" t="s">
         <v>67</v>
       </c>
-      <c r="L12" t="s">
+      <c r="L13" t="s">
         <v>68</v>
       </c>
-      <c r="M12" t="s">
+      <c r="M13" t="s">
         <v>163</v>
       </c>
-      <c r="N12" t="s">
+      <c r="N13" t="s">
         <v>70</v>
       </c>
-      <c r="O12" t="s">
+      <c r="O13" t="s">
         <v>71</v>
       </c>
-      <c r="P12" t="s">
+      <c r="P13" t="s">
         <v>68</v>
       </c>
-      <c r="Q12" t="s">
+      <c r="Q13" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>165</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B14" t="s">
         <v>167</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C14" t="s">
         <v>168</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D14" t="s">
         <v>169</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E14" t="s">
         <v>74</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F14" t="s">
         <v>166</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G14" t="s">
         <v>170</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H14" t="s">
         <v>171</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I14" t="s">
         <v>172</v>
       </c>
-      <c r="J13" t="s">
+      <c r="J14" t="s">
         <v>173</v>
       </c>
-      <c r="K13" t="s">
+      <c r="K14" t="s">
         <v>174</v>
       </c>
-      <c r="L13" t="s">
+      <c r="L14" t="s">
         <v>175</v>
       </c>
-      <c r="M13" t="s">
+      <c r="M14" t="s">
         <v>176</v>
       </c>
-      <c r="N13" t="s">
+      <c r="N14" t="s">
         <v>177</v>
       </c>
-      <c r="O13" t="s">
+      <c r="O14" t="s">
         <v>178</v>
       </c>
-      <c r="P13" t="s">
+      <c r="P14" t="s">
         <v>179</v>
       </c>
-      <c r="Q13" t="s">
+      <c r="Q14" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>181</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B15" t="s">
         <v>91</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C15" t="s">
         <v>183</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D15" t="s">
         <v>184</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E15" t="s">
         <v>91</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F15" t="s">
         <v>182</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G15" t="s">
         <v>185</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H15" t="s">
         <v>186</v>
       </c>
-      <c r="I14" t="s">
+      <c r="I15" t="s">
         <v>187</v>
       </c>
-      <c r="J14" t="s">
+      <c r="J15" t="s">
         <v>188</v>
       </c>
-      <c r="K14" t="s">
+      <c r="K15" t="s">
         <v>91</v>
       </c>
-      <c r="L14" t="s">
+      <c r="L15" t="s">
         <v>189</v>
       </c>
-      <c r="M14" t="s">
+      <c r="M15" t="s">
         <v>91</v>
       </c>
-      <c r="N14" t="s">
+      <c r="N15" t="s">
         <v>190</v>
       </c>
-      <c r="O14" t="s">
+      <c r="O15" t="s">
         <v>91</v>
       </c>
-      <c r="P14" t="s">
+      <c r="P15" t="s">
         <v>91</v>
       </c>
-      <c r="Q14" t="s">
+      <c r="Q15" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>192</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>194</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C16" t="s">
         <v>195</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D16" t="s">
         <v>196</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E16" t="s">
         <v>197</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F16" t="s">
         <v>193</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H16" t="s">
         <v>199</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I16" t="s">
         <v>200</v>
       </c>
-      <c r="J15" s="3" t="s">
+      <c r="J16" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="K15" s="3" t="s">
+      <c r="K16" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="L15" s="3" t="s">
+      <c r="L16" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="M15" s="3" t="s">
+      <c r="M16" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="N15" s="3" t="s">
+      <c r="N16" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="O15" s="3" t="s">
+      <c r="O16" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="P15" s="3" t="s">
+      <c r="P16" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="Q15" s="3" t="s">
+      <c r="Q16" s="3" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="R16" s="4" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>209</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B17" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="C17" t="s">
+        <v>229</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="H17" t="s">
         <v>228</v>
       </c>
-      <c r="C16" t="s">
-        <v>230</v>
-      </c>
-      <c r="E16" s="4" t="s">
+      <c r="L17" t="s">
+        <v>225</v>
+      </c>
+      <c r="N17" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>311</v>
+      </c>
+      <c r="B18" t="s">
+        <v>210</v>
+      </c>
+      <c r="C18" t="s">
+        <v>211</v>
+      </c>
+      <c r="D18" t="s">
+        <v>212</v>
+      </c>
+      <c r="E18" t="s">
+        <v>213</v>
+      </c>
+      <c r="G18" t="s">
+        <v>214</v>
+      </c>
+      <c r="H18" t="s">
+        <v>215</v>
+      </c>
+      <c r="I18" t="s">
+        <v>216</v>
+      </c>
+      <c r="J18" t="s">
+        <v>217</v>
+      </c>
+      <c r="K18" t="s">
+        <v>218</v>
+      </c>
+      <c r="L18" t="s">
+        <v>219</v>
+      </c>
+      <c r="M18" t="s">
+        <v>220</v>
+      </c>
+      <c r="N18" t="s">
+        <v>221</v>
+      </c>
+      <c r="O18" t="s">
+        <v>222</v>
+      </c>
+      <c r="P18" t="s">
+        <v>223</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>224</v>
+      </c>
+      <c r="R18" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>254</v>
+      </c>
+      <c r="B19" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>255</v>
+      </c>
+      <c r="B20" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>256</v>
+      </c>
+      <c r="B21" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>257</v>
+      </c>
+      <c r="B22" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>258</v>
+      </c>
+      <c r="B23" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>232</v>
+      </c>
+      <c r="B24" t="s">
         <v>231</v>
       </c>
-      <c r="H16" t="s">
-        <v>229</v>
-      </c>
-      <c r="L16" t="s">
-        <v>226</v>
-      </c>
-      <c r="N16" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>210</v>
-      </c>
-      <c r="B17" t="s">
-        <v>211</v>
-      </c>
-      <c r="C17" t="s">
-        <v>212</v>
-      </c>
-      <c r="D17" t="s">
-        <v>213</v>
-      </c>
-      <c r="E17" t="s">
-        <v>214</v>
-      </c>
-      <c r="G17" t="s">
-        <v>215</v>
-      </c>
-      <c r="H17" t="s">
-        <v>216</v>
-      </c>
-      <c r="I17" t="s">
-        <v>217</v>
-      </c>
-      <c r="J17" t="s">
-        <v>218</v>
-      </c>
-      <c r="K17" t="s">
-        <v>219</v>
-      </c>
-      <c r="L17" t="s">
-        <v>220</v>
-      </c>
-      <c r="M17" t="s">
-        <v>221</v>
-      </c>
-      <c r="N17" t="s">
-        <v>222</v>
-      </c>
-      <c r="O17" t="s">
-        <v>223</v>
-      </c>
-      <c r="P17" t="s">
-        <v>224</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>255</v>
-      </c>
-      <c r="B18" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>256</v>
-      </c>
-      <c r="B19" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>257</v>
-      </c>
-      <c r="B20" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>258</v>
-      </c>
-      <c r="B21" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>259</v>
-      </c>
-      <c r="B22" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>233</v>
       </c>
-      <c r="B23" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="B25" t="s">
         <v>234</v>
       </c>
-      <c r="B24" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>239</v>
-      </c>
-      <c r="B25" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>238</v>
       </c>
       <c r="B26" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="B27" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>295</v>
+      </c>
+      <c r="B28" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>296</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B29" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>297</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B30" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>298</v>
-      </c>
-      <c r="B29" t="s">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>243</v>
+      </c>
+      <c r="B31" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>245</v>
+      </c>
+      <c r="B32" t="s">
         <v>244</v>
       </c>
-      <c r="B30" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>249</v>
+      </c>
+      <c r="B33" t="s">
         <v>246</v>
       </c>
-      <c r="B31" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    </row>
+    <row r="34" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>250</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B34" s="5" t="s">
         <v>247</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>251</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>252</v>
-      </c>
-      <c r="B34" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="B35" t="s">
-        <v>264</v>
+        <v>248</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="B36" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B37" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B38" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B39" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B40" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="B41" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B42" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>300</v>
+        <v>277</v>
       </c>
       <c r="B43" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -2451,142 +2476,353 @@
         <v>299</v>
       </c>
       <c r="B44" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="B45" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B46" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B47" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B48" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B49" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>304</v>
+      </c>
+      <c r="B50" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>305</v>
+      </c>
+      <c r="B51" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>306</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B52" s="5" t="s">
         <v>286</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>307</v>
-      </c>
-      <c r="B51" s="5" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>308</v>
-      </c>
-      <c r="B52" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="B53" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>308</v>
+      </c>
+      <c r="B54" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>309</v>
+      </c>
+      <c r="B55" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" ht="120" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
         <v>310</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B56" s="5" t="s">
         <v>289</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="135" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>311</v>
-      </c>
-      <c r="B55" s="5" t="s">
-        <v>290</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="B15" r:id="rId1" display="https://exerzitien" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="G15" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="J15" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="K15" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="L15" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="M15" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="N15" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="O15" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="P15" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="Q15" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="B16" r:id="rId11" xr:uid="{787A4DE5-335B-4B11-A6F3-1E6F83DC3CEE}"/>
-    <hyperlink ref="E16" r:id="rId12" xr:uid="{BCA7FA4C-37A2-4ED7-9F0D-002142A07A10}"/>
+    <hyperlink ref="B16" r:id="rId1" display="https://exerzitien" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="G16" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="J16" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="K16" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="L16" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="M16" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="N16" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="O16" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="P16" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="Q16" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="B17" r:id="rId11" xr:uid="{787A4DE5-335B-4B11-A6F3-1E6F83DC3CEE}"/>
+    <hyperlink ref="E17" r:id="rId12" xr:uid="{BCA7FA4C-37A2-4ED7-9F0D-002142A07A10}"/>
+    <hyperlink ref="R16" r:id="rId13" xr:uid="{31BFF9C6-9435-43E8-8F31-E093CDB89BE1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId13"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId14"/>
   <tableParts count="1">
-    <tablePart r:id="rId14"/>
+    <tablePart r:id="rId15"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A2:A4"/>
+  <dimension ref="A2:F19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>291</v>
+      </c>
+      <c r="D2" t="s">
+        <v>294</v>
+      </c>
+      <c r="E2" t="s">
+        <v>192</v>
+      </c>
+      <c r="F2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F3" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>293</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>294</v>
+      <c r="D4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" t="s">
+        <v>195</v>
+      </c>
+      <c r="F4" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" t="s">
+        <v>196</v>
+      </c>
+      <c r="F5" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" t="s">
+        <v>197</v>
+      </c>
+      <c r="F6" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="F8" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" t="s">
+        <v>199</v>
+      </c>
+      <c r="F9" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" t="s">
+        <v>200</v>
+      </c>
+      <c r="F10" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="F11" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="F12" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="F13" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="F14" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D15" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="F15" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="F16" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="17" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="F17" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="18" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D18" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="F18" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="19" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D19" t="s">
+        <v>312</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="F19" t="s">
+        <v>316</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E3" r:id="rId1" display="https://exerzitien" xr:uid="{334610EE-AE7A-4FB5-808C-09410BEBA6C6}"/>
+    <hyperlink ref="E8" r:id="rId2" xr:uid="{617D7274-0DEC-4994-A59D-27B10CF96B56}"/>
+    <hyperlink ref="E11" r:id="rId3" xr:uid="{3BC45541-A0EF-4FF9-A021-3FB7D18C0240}"/>
+    <hyperlink ref="E12" r:id="rId4" xr:uid="{EF8655C5-A9F7-4595-B65A-4636D97D2C69}"/>
+    <hyperlink ref="E13" r:id="rId5" xr:uid="{45F0088F-BEFC-4A58-8D01-13E91C5A7C72}"/>
+    <hyperlink ref="E14" r:id="rId6" xr:uid="{7458D400-607A-4CF4-9094-67837CAE9A8B}"/>
+    <hyperlink ref="E15" r:id="rId7" xr:uid="{671C83DA-5E9C-4F2F-B92A-D33098304811}"/>
+    <hyperlink ref="E16" r:id="rId8" xr:uid="{8874929A-D30A-4261-AAA7-EB9D9FC62B21}"/>
+    <hyperlink ref="E17" r:id="rId9" xr:uid="{76A07235-FA82-4263-BADD-FE54F8CDDA1A}"/>
+    <hyperlink ref="E18" r:id="rId10" xr:uid="{10ED4BBB-8938-4873-97F8-BC48AFEC3D59}"/>
+    <hyperlink ref="E19" r:id="rId11" xr:uid="{FAD7111C-3364-46F2-BE58-92386FF9900A}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>